<commit_message>
chore(data-release): publish site data 2026-10-28 11:51:53 UTC
</commit_message>
<xml_diff>
--- a/countries/be/2020-2025.xlsx
+++ b/countries/be/2020-2025.xlsx
@@ -34283,22 +34283,22 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>D045</t>
+          <t>D040</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Echinococcosis</t>
+          <t>Rubella</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>包虫病</t>
+          <t>风疹</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
@@ -34312,17 +34312,17 @@
         </is>
       </c>
       <c r="N235" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="O235" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="R235" t="n">
-        <v>0.3061588183562282</v>
+        <v>0</v>
       </c>
       <c r="U235" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_ECHI_ANNUAL</t>
+          <t>SER_BE_ECDC_RUBE_ANNUAL</t>
         </is>
       </c>
       <c r="AA235" t="inlineStr">
@@ -34342,7 +34342,7 @@
       </c>
       <c r="AS235" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_ECHI_ANNUAL</t>
+          <t>SER_BE_ECDC_RUBE_ANNUAL</t>
         </is>
       </c>
       <c r="AT235" t="n">
@@ -34427,22 +34427,22 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>D092</t>
+          <t>D045</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Campylobacteriosis</t>
+          <t>Echinococcosis</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>弯曲杆菌病</t>
+          <t>包虫病</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Parasitic</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
@@ -34456,17 +34456,17 @@
         </is>
       </c>
       <c r="N236" t="n">
-        <v>7454</v>
+        <v>36</v>
       </c>
       <c r="O236" t="n">
-        <v>7454</v>
+        <v>36</v>
       </c>
       <c r="R236" t="n">
-        <v>63.39188422298125</v>
+        <v>0.3061588183562282</v>
       </c>
       <c r="U236" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_CAMP_ANNUAL</t>
+          <t>SER_BE_ECDC_ECHI_ANNUAL</t>
         </is>
       </c>
       <c r="AA236" t="inlineStr">
@@ -34486,7 +34486,7 @@
       </c>
       <c r="AS236" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_CAMP_ANNUAL</t>
+          <t>SER_BE_ECDC_ECHI_ANNUAL</t>
         </is>
       </c>
       <c r="AT236" t="n">
@@ -34571,17 +34571,17 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>D105</t>
+          <t>D092</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Shigellosis</t>
+          <t>Campylobacteriosis</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>志贺菌病</t>
+          <t>弯曲杆菌病</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -34600,17 +34600,17 @@
         </is>
       </c>
       <c r="N237" t="n">
-        <v>479</v>
+        <v>7454</v>
       </c>
       <c r="O237" t="n">
-        <v>479</v>
+        <v>7454</v>
       </c>
       <c r="R237" t="n">
-        <v>4.073613166462037</v>
+        <v>63.39188422298125</v>
       </c>
       <c r="U237" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_SHIG_ANNUAL</t>
+          <t>SER_BE_ECDC_CAMP_ANNUAL</t>
         </is>
       </c>
       <c r="AA237" t="inlineStr">
@@ -34630,7 +34630,7 @@
       </c>
       <c r="AS237" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_SHIG_ANNUAL</t>
+          <t>SER_BE_ECDC_CAMP_ANNUAL</t>
         </is>
       </c>
       <c r="AT237" t="n">
@@ -34715,17 +34715,17 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D105</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Shigellosis</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>志贺菌病</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -34744,17 +34744,17 @@
         </is>
       </c>
       <c r="N238" t="n">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="O238" t="n">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="R238" t="n">
-        <v>3.512321999475618</v>
+        <v>4.073613166462037</v>
       </c>
       <c r="U238" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BE_ECDC_SHIG_ANNUAL</t>
         </is>
       </c>
       <c r="AA238" t="inlineStr">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="AS238" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BE_ECDC_SHIG_ANNUAL</t>
         </is>
       </c>
       <c r="AT238" t="n">
@@ -34859,17 +34859,17 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>D108</t>
+          <t>D107</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Listeriosis</t>
+          <t>Legionellosis</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>李斯特菌病</t>
+          <t>军团菌病</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -34888,17 +34888,17 @@
         </is>
       </c>
       <c r="N239" t="n">
-        <v>101</v>
+        <v>413</v>
       </c>
       <c r="O239" t="n">
-        <v>101</v>
+        <v>413</v>
       </c>
       <c r="R239" t="n">
-        <v>0.8589455737216403</v>
+        <v>3.512321999475618</v>
       </c>
       <c r="U239" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_LIST_ANNUAL</t>
+          <t>SER_BE_ECDC_LEGI_ANNUAL</t>
         </is>
       </c>
       <c r="AA239" t="inlineStr">
@@ -34918,7 +34918,7 @@
       </c>
       <c r="AS239" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_LIST_ANNUAL</t>
+          <t>SER_BE_ECDC_LEGI_ANNUAL</t>
         </is>
       </c>
       <c r="AT239" t="n">
@@ -35003,17 +35003,17 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>D114</t>
+          <t>D108</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Salmonellosis</t>
+          <t>Listeriosis</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>沙门氏菌病</t>
+          <t>李斯特菌病</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -35032,17 +35032,17 @@
         </is>
       </c>
       <c r="N240" t="n">
-        <v>2554</v>
+        <v>101</v>
       </c>
       <c r="O240" t="n">
-        <v>2554</v>
+        <v>101</v>
       </c>
       <c r="R240" t="n">
-        <v>21.72026728005019</v>
+        <v>0.8589455737216403</v>
       </c>
       <c r="U240" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_SALM_ANNUAL</t>
+          <t>SER_BE_ECDC_LIST_ANNUAL</t>
         </is>
       </c>
       <c r="AA240" t="inlineStr">
@@ -35062,7 +35062,7 @@
       </c>
       <c r="AS240" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_SALM_ANNUAL</t>
+          <t>SER_BE_ECDC_LIST_ANNUAL</t>
         </is>
       </c>
       <c r="AT240" t="n">
@@ -35147,17 +35147,17 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>D115</t>
+          <t>D114</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Shiga toxin-producing Escherichia coli infection</t>
+          <t>Salmonellosis</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>产志贺毒素大肠杆菌感染</t>
+          <t>沙门氏菌病</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -35176,17 +35176,17 @@
         </is>
       </c>
       <c r="N241" t="n">
-        <v>1039</v>
+        <v>2554</v>
       </c>
       <c r="O241" t="n">
-        <v>1039</v>
+        <v>2554</v>
       </c>
       <c r="R241" t="n">
-        <v>8.836083674225586</v>
+        <v>21.72026728005019</v>
       </c>
       <c r="U241" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_STEC_ANNUAL</t>
+          <t>SER_BE_ECDC_SALM_ANNUAL</t>
         </is>
       </c>
       <c r="AA241" t="inlineStr">
@@ -35206,7 +35206,7 @@
       </c>
       <c r="AS241" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_STEC_ANNUAL</t>
+          <t>SER_BE_ECDC_SALM_ANNUAL</t>
         </is>
       </c>
       <c r="AT241" t="n">
@@ -35291,22 +35291,22 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>D122</t>
+          <t>D115</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Trichinellosis</t>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>旋毛虫病</t>
+          <t>产志贺毒素大肠杆菌感染</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
@@ -35320,17 +35320,17 @@
         </is>
       </c>
       <c r="N242" t="n">
-        <v>0</v>
+        <v>1039</v>
       </c>
       <c r="O242" t="n">
-        <v>0</v>
+        <v>1039</v>
       </c>
       <c r="R242" t="n">
-        <v>0</v>
+        <v>8.836083674225586</v>
       </c>
       <c r="U242" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_TRIC_ANNUAL</t>
+          <t>SER_BE_ECDC_STEC_ANNUAL</t>
         </is>
       </c>
       <c r="AA242" t="inlineStr">
@@ -35350,7 +35350,7 @@
       </c>
       <c r="AS242" t="inlineStr">
         <is>
-          <t>SER_BE_ECDC_TRIC_ANNUAL</t>
+          <t>SER_BE_ECDC_STEC_ANNUAL</t>
         </is>
       </c>
       <c r="AT242" t="n">
@@ -35392,6 +35392,150 @@
         </is>
       </c>
       <c r="BC242" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>be</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>be</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>0</v>
+      </c>
+      <c r="O243" t="n">
+        <v>0</v>
+      </c>
+      <c r="R243" t="n">
+        <v>0</v>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>SER_BE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO243" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP243" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS243" t="inlineStr">
+        <is>
+          <t>SER_BE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT243" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV243" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW243" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Belgium Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX243" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY243" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ243" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA243" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Belgium Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB243" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC243" t="inlineStr">
         <is>
           <t>official_ecdc_rest_aggregate</t>
         </is>
@@ -35513,7 +35657,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10">
@@ -35523,7 +35667,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">

</xml_diff>